<commit_message>
bump xlwings version to 0.36.6 and add object handle tests
</commit_message>
<xml_diff>
--- a/tests/e2e_custom_functions.xlsx
+++ b/tests/e2e_custom_functions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10609"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/dev/xlwings-server/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A564224-9359-414F-B13D-0CBD833E7293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA1B36F-02DA-5341-9468-C282CB9F5353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="900" yWindow="780" windowWidth="33300" windowHeight="21360" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="9">
+  <futureMetadata name="XLRICHVALUE" count="10">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -111,13 +111,20 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="9"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="9">
+  <valueMetadata count="10">
     <bk>
       <rc t="2" v="0"/>
     </bk>
@@ -145,12 +152,15 @@
     <bk>
       <rc t="2" v="8"/>
     </bk>
+    <bk>
+      <rc t="2" v="9"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="144">
   <si>
     <t>epected</t>
   </si>
@@ -579,6 +589,9 @@
   </si>
   <si>
     <t>required_roles</t>
+  </si>
+  <si>
+    <t>nested_object_call</t>
   </si>
 </sst>
 </file>
@@ -839,13 +852,13 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="10">
   <rv s="0">
     <fb>25568</fb>
     <v>0</v>
   </rv>
   <rv s="0">
-    <fb>27805.546099537041</fb>
+    <fb>27805.546099537038</fb>
     <v>0</v>
   </rv>
   <rv s="0">
@@ -870,9 +883,21 @@
   </rv>
   <rv s="1">
     <v>DataFrame</v>
+    <v>3</v>
     <v>Generic</v>
     <v>A [int64], B [int64], C [int64]</v>
     <v>RangeIndex: 5 entries, 0 to 4</v>
+    <v>040068ef-e37e-46f1-8d64-6bc59f763a94</v>
+    <v>(5, 3)</v>
+    <v>DataFrame</v>
+  </rv>
+  <rv s="1">
+    <v>DataFrame</v>
+    <v>3</v>
+    <v>Generic</v>
+    <v>A [int64], B [int64], C [int64]</v>
+    <v>RangeIndex: 5 entries, 0 to 4</v>
+    <v>08011596-1b8e-43e8-8af4-d4602a69c679</v>
     <v>(5, 3)</v>
     <v>DataFrame</v>
   </rv>
@@ -889,9 +914,11 @@
   </s>
   <s t="_entity">
     <k n="_DisplayString" t="s"/>
+    <k n="_Flags" t="spb"/>
     <k n="_Icon" t="s"/>
     <k n="Columns" t="s"/>
     <k n="Index" t="s"/>
+    <k n="object_handle_cache_key" t="s"/>
     <k n="Shape" t="s"/>
     <k n="Type" t="s"/>
   </s>
@@ -903,11 +930,19 @@
 
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
-  <spbData count="2">
+  <spbData count="4">
     <spb s="0">
       <v>1</v>
     </spb>
     <spb s="0">
+      <v>2</v>
+    </spb>
+    <spb s="1">
+      <v>0</v>
+      <v>0</v>
+      <v>0</v>
+    </spb>
+    <spb s="2">
       <v>2</v>
     </spb>
   </spbData>
@@ -915,9 +950,17 @@
 </file>
 
 <file path=xl/richData/rdsupportingpropertybagstructure.xml><?xml version="1.0" encoding="utf-8"?>
-<spbStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="1">
+<spbStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="3">
   <s>
     <k n="_Self" t="i"/>
+  </s>
+  <s>
+    <k n="ShowInCardView" t="b"/>
+    <k n="ShowInDotNotation" t="b"/>
+    <k n="ShowInAutoComplete" t="b"/>
+  </s>
+  <s>
+    <k n="object_handle_cache_key" t="spb"/>
   </s>
 </spbStructures>
 </file>
@@ -934,7 +977,7 @@
   </richProperties>
   <richStyles>
     <rSty dxfid="0">
-      <rpv i="0">m/d/yyyy</rpv>
+      <rpv i="0">m/d/yy</rpv>
     </rSty>
     <rSty dxfid="0">
       <rpv i="0">yyyy-m-d</rpv>
@@ -1442,6 +1485,7 @@
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_PARSE_DATES_NAMES</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_PARSE_DATES_TRUE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_READ_2DLIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGS_DEV_READ_CACHE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_READ_DATE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_READ_DATE_NPARRAY</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_READ_DATES_AS1</we:customFunctionIds>
@@ -1521,6 +1565,7 @@
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_VIEW</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_VOLATILE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_WRITE_2DLIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGS_DEV_WRITE_CACHE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_WRITE_DATE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_WRITE_DATETIME</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGS_DEV_WRITE_DF_0HEADER_0INDEX</we:customFunctionIds>
@@ -1565,7 +1610,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P409"/>
+  <dimension ref="A1:P412"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
@@ -1835,7 +1880,7 @@
       </c>
       <c r="G24" s="16" cm="1" vm="2">
         <f t="array" ref="G24">_xldudf_XLWINGS_DEV_WRITE_DATETIME()</f>
-        <v>27805.546099537041</v>
+        <v>27805.546099537038</v>
       </c>
       <c r="H24" t="b">
         <f>F24=G24</f>
@@ -8154,7 +8199,7 @@
       </c>
     </row>
     <row r="407" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="F407" t="e" cm="1" vm="8">
+      <c r="F407" t="e" cm="1" vm="9">
         <f t="array" ref="F407">_xldudf_XLWINGS_DEV_GET_DF()</f>
         <v>#VALUE!</v>
       </c>
@@ -8167,12 +8212,29 @@
       <c r="B409" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="F409" t="e" cm="1" vm="9">
+      <c r="F409" t="e" cm="1" vm="10">
         <f t="array" ref="F409">_xldudf_XLWINGS_DEV_REQUIRED_ROLES()</f>
         <v>#VALUE!</v>
       </c>
       <c r="G409" s="2" t="b">
         <f>ISERROR(F409)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="412" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A412" t="b">
+        <f>G412</f>
+        <v>1</v>
+      </c>
+      <c r="B412" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F412" t="str" cm="1">
+        <f t="array" ref="F412">_xldudf_XLWINGS_DEV_READ_CACHE(_xldudf_XLWINGS_DEV_WRITE_CACHE("A"), _xldudf_XLWINGS_DEV_WRITE_CACHE("B"))</f>
+        <v>SUCCESS</v>
+      </c>
+      <c r="G412" s="2" t="b">
+        <f>F412="SUCCESS"</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>